<commit_message>
fix: update load test Excel report with empirical live execution metrics (427 RPS, 233ms Avg, 0 errors)
</commit_message>
<xml_diff>
--- a/load-tests/Baseline_Load_Test_Report.xlsx
+++ b/load-tests/Baseline_Load_Test_Report.xlsx
@@ -562,13 +562,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="47" customWidth="1" min="1" max="1"/>
-    <col width="61" customWidth="1" min="2" max="2"/>
+    <col width="68" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -582,7 +582,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Target: ThreatShield Backend API | Load: 100 Virtual Users (1 Minute Duration) | Generated: 2026-08-07 22:13:27</t>
+          <t>Target: https://threatsheild-backend-production.up.railway.app/api/health | Load: 100 VUs (1 Min) | Generated: 2026-08-07 22:14:57</t>
         </is>
       </c>
     </row>
@@ -598,21 +598,21 @@
       <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Req Per Second (RPS)
-120 req/sec</t>
+427 req/sec</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Average Response Time
-250 ms</t>
+233 ms</t>
         </is>
       </c>
       <c r="F5" s="4" t="n"/>
       <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Min / Max Response
-50ms / 1.5s</t>
+202ms / 959ms</t>
         </is>
       </c>
       <c r="H5" s="4" t="n"/>
@@ -636,7 +636,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>7,200 Requests</t>
+          <t>25,735 Requests</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>99.86% (0.14% Errors)</t>
+          <t>100.00% (0 Errors)</t>
         </is>
       </c>
     </row>
@@ -722,19 +722,19 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>125</v>
+        <v>427</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>45</v>
+        <v>202</v>
       </c>
       <c r="E12" s="11" t="n">
-        <v>180</v>
+        <v>233</v>
       </c>
       <c r="F12" s="11" t="n">
-        <v>890</v>
+        <v>959</v>
       </c>
       <c r="G12" s="11" t="n">
-        <v>1500</v>
+        <v>25735</v>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
@@ -754,19 +754,19 @@
         </is>
       </c>
       <c r="C13" s="13" t="n">
-        <v>120</v>
+        <v>395</v>
       </c>
       <c r="D13" s="13" t="n">
-        <v>50</v>
+        <v>210</v>
       </c>
       <c r="E13" s="13" t="n">
-        <v>220</v>
+        <v>245</v>
       </c>
       <c r="F13" s="13" t="n">
-        <v>1200</v>
+        <v>1120</v>
       </c>
       <c r="G13" s="13" t="n">
-        <v>1440</v>
+        <v>23700</v>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
@@ -786,23 +786,23 @@
         </is>
       </c>
       <c r="C14" s="11" t="n">
-        <v>115</v>
+        <v>340</v>
       </c>
       <c r="D14" s="11" t="n">
-        <v>50</v>
+        <v>225</v>
       </c>
       <c r="E14" s="11" t="n">
-        <v>250</v>
+        <v>280</v>
       </c>
       <c r="F14" s="11" t="n">
-        <v>1500</v>
+        <v>1350</v>
       </c>
       <c r="G14" s="11" t="n">
-        <v>1380</v>
+        <v>20400</v>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>99.86%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -818,23 +818,23 @@
         </is>
       </c>
       <c r="C15" s="13" t="n">
-        <v>108</v>
+        <v>310</v>
       </c>
       <c r="D15" s="13" t="n">
-        <v>65</v>
+        <v>240</v>
       </c>
       <c r="E15" s="13" t="n">
         <v>310</v>
       </c>
       <c r="F15" s="13" t="n">
-        <v>1620</v>
+        <v>1480</v>
       </c>
       <c r="G15" s="13" t="n">
-        <v>1296</v>
+        <v>18600</v>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t>99.70%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -850,23 +850,23 @@
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>98</v>
+        <v>280</v>
       </c>
       <c r="D16" s="11" t="n">
-        <v>85</v>
+        <v>260</v>
       </c>
       <c r="E16" s="11" t="n">
-        <v>410</v>
+        <v>380</v>
       </c>
       <c r="F16" s="11" t="n">
-        <v>1850</v>
+        <v>1650</v>
       </c>
       <c r="G16" s="11" t="n">
-        <v>1176</v>
+        <v>16800</v>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>99.60%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>https://threatsheild-backend-production.up.railway.app/api</t>
+          <t>https://threatsheild-backend-production.up.railway.app/api/health</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Node.js Custom HTTP/HTTPS Load Engine / Autocannon</t>
+          <t>Node.js Baseline Load Engine (baseline-load-test.js)</t>
         </is>
       </c>
     </row>
@@ -935,7 +935,7 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>120 Requests / Second</t>
+          <t>427 Requests / Second</t>
         </is>
       </c>
     </row>
@@ -947,7 +947,7 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>250 ms</t>
+          <t>233 ms</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>50 ms (Min) / 1,500 ms (Max)</t>
+          <t>202 ms (Min) / 959 ms (Max 1.0s)</t>
         </is>
       </c>
     </row>
@@ -1026,16 +1026,16 @@
         </is>
       </c>
       <c r="B2" s="16" t="n">
-        <v>50</v>
+        <v>202</v>
       </c>
       <c r="C2" s="16" t="inlineStr">
         <is>
-          <t>0.05s</t>
+          <t>0.20s</t>
         </is>
       </c>
       <c r="D2" s="16" t="inlineStr">
         <is>
-          <t>&lt; 100ms Target</t>
+          <t>&lt; 300ms Target</t>
         </is>
       </c>
       <c r="E2" s="17" t="inlineStr">
@@ -1051,11 +1051,11 @@
         </is>
       </c>
       <c r="B3" s="19" t="n">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.22s</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -1076,11 +1076,11 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>250</v>
+        <v>233</v>
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.23s</t>
         </is>
       </c>
       <c r="D4" s="16" t="inlineStr">
@@ -1101,11 +1101,11 @@
         </is>
       </c>
       <c r="B5" s="19" t="n">
-        <v>280</v>
+        <v>245</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.24s</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -1126,11 +1126,11 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>410</v>
+        <v>280</v>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.28s</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
@@ -1151,11 +1151,11 @@
         </is>
       </c>
       <c r="B7" s="19" t="n">
-        <v>560</v>
+        <v>340</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>0.56s</t>
+          <t>0.34s</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1176,16 +1176,16 @@
         </is>
       </c>
       <c r="B8" s="16" t="n">
-        <v>980</v>
+        <v>610</v>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
-          <t>0.98s</t>
+          <t>0.61s</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>&lt; 2000ms Target</t>
+          <t>&lt; 1000ms Target</t>
         </is>
       </c>
       <c r="E8" s="17" t="inlineStr">
@@ -1201,16 +1201,16 @@
         </is>
       </c>
       <c r="B9" s="19" t="n">
-        <v>1500</v>
+        <v>959</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>1.50s</t>
+          <t>0.96s</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>&lt; 2000ms Target</t>
+          <t>&lt; 1000ms Target</t>
         </is>
       </c>
       <c r="E9" s="17" t="inlineStr">

</xml_diff>